<commit_message>
Update: fixed wrong entry in manifest
</commit_message>
<xml_diff>
--- a/data/initial_inspection_samples/Initial_inspection_samples_manifest.xlsx
+++ b/data/initial_inspection_samples/Initial_inspection_samples_manifest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\badho\Desktop\Projects\PrecisionFarming\data\initial_inspection_samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E3D2AE-5ADE-47CA-B975-6DD28C5FBF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E442E4-34FD-4D6E-B3D9-D70FA65768ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13920" xr2:uid="{9711B223-4ED4-41C5-884A-5F9FED30802F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="33">
   <si>
     <t>ImageID</t>
   </si>
@@ -132,6 +132,12 @@
   </si>
   <si>
     <t>wide arial shot makes hard to see the leaves without zooming</t>
+  </si>
+  <si>
+    <t>Field-Erftstadt/26_07_07</t>
+  </si>
+  <si>
+    <t>https://hshl.sciebo.de/s/g2QCsQzRqABPYmd?dir=%2FField-Erftstadt%2F26_07_07</t>
   </si>
 </sst>
 </file>
@@ -179,7 +185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -193,12 +199,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -212,17 +212,17 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_([$€-2]\ * #,##0.00_);_([$€-2]\ * \(#,##0.00\);_([$€-2]\ * &quot;-&quot;??_);_(@_)"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -250,16 +250,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11FA4875-8DC1-47A3-A418-87E884128461}" name="Table1" displayName="Table1" ref="A1:H10" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11FA4875-8DC1-47A3-A418-87E884128461}" name="Table1" displayName="Table1" ref="A1:H10" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="A1:H10" xr:uid="{11FA4875-8DC1-47A3-A418-87E884128461}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{6A941C9D-2713-4DCB-A4EE-470D8B65CD27}" name="ImageID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{CEA0A04D-E4FC-4ED3-A9EB-34A5DD80D828}" name="Filename" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{3764309B-A057-4959-9734-3AFB38B13B55}" name="Source" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{DEF7FDE9-7AC8-425D-B966-E1CB01DEC4F0}" name="Dimention (wxh)" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{C81320DA-5959-4F05-ADF1-1FE4784CCAD5}" name="Quality" dataDxfId="5" dataCellStyle="Currency"/>
-    <tableColumn id="6" xr3:uid="{1C99875D-E024-442A-B5EA-659246B404AB}" name="Is Good for Model Training" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{FF3989E5-4695-4B95-B0A0-3BA37FB858A5}" name="Dir Link" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{6A941C9D-2713-4DCB-A4EE-470D8B65CD27}" name="ImageID" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{CEA0A04D-E4FC-4ED3-A9EB-34A5DD80D828}" name="Filename" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{3764309B-A057-4959-9734-3AFB38B13B55}" name="Source" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{DEF7FDE9-7AC8-425D-B966-E1CB01DEC4F0}" name="Dimention (wxh)" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{C81320DA-5959-4F05-ADF1-1FE4784CCAD5}" name="Quality" dataDxfId="3" dataCellStyle="Currency"/>
+    <tableColumn id="6" xr3:uid="{1C99875D-E024-442A-B5EA-659246B404AB}" name="Is Good for Model Training" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{FF3989E5-4695-4B95-B0A0-3BA37FB858A5}" name="Dir Link" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{688078B1-1F97-4A9A-B47B-884A6C07FAC9}" name="Reasoning" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -629,7 +629,7 @@
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -641,7 +641,7 @@
       <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -719,7 +719,7 @@
       <c r="F5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -745,7 +745,7 @@
       <c r="F6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -771,7 +771,7 @@
       <c r="F7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H7" s="2" t="s">
@@ -797,14 +797,14 @@
       <c r="F8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="72.900000000000006" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -812,7 +812,7 @@
         <v>26</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>24</v>
@@ -823,8 +823,8 @@
       <c r="F9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>16</v>
+      <c r="G9" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>29</v>

</xml_diff>